<commit_message>
docs: perbarui petunjuk pengisian template upload Excel sesuai logika realisasi bulanan mentah
</commit_message>
<xml_diff>
--- a/data/template_upload.xlsx
+++ b/data/template_upload.xlsx
@@ -1,14 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Data Realisasi" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Petunjuk Pengisian" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Realisasi" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Petunjuk Pengisian" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,10 +17,18 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
@@ -75,12 +82,27 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -96,43 +118,47 @@
       <bottom style="thin">
         <color rgb="00D9D9D9"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -509,151 +535,151 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>tahun</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>nama_opd</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>penanggungjawab</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>kode_rekening</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>jenis_belanja</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>bulan</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>pagu_anggaran</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>realisasi</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="3" t="n">
         <v>2025</v>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>Badan Keuangan dan Aset Daerah (BKAD)</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>Sekretariat</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>5.02.01.2.01.0001</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>Penyusunan Dokumen Perencanaan Perangkat Daerah</t>
         </is>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="F2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="G2" s="4" t="n">
+      <c r="G2" s="5" t="n">
         <v>16342500</v>
       </c>
-      <c r="H2" s="4" t="n">
+      <c r="H2" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="3" t="n">
         <v>2025</v>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Badan Keuangan dan Aset Daerah (BKAD)</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Sekretariat</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>5.02.01.2.01.0001</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>Penyusunan Dokumen Perencanaan Perangkat Daerah</t>
         </is>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="F3" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G3" s="4" t="n">
+      <c r="G3" s="5" t="n">
         <v>16342500</v>
       </c>
-      <c r="H3" s="4" t="n">
+      <c r="H3" s="5" t="n">
         <v>2440000</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="3" t="n">
         <v>2025</v>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Badan Keuangan dan Aset Daerah (BKAD)</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Bidang Anggaran</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>5.02.02.2.01.0001</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Koordinasi dan Penyusunan KUA dan PPAS</t>
         </is>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="F4" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="G4" s="4" t="n">
+      <c r="G4" s="5" t="n">
         <v>325936500</v>
       </c>
-      <c r="H4" s="4" t="n">
+      <c r="H4" s="5" t="n">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -674,343 +700,343 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>PETUNJUK PENGISIAN TEMPLATE DATA REALISASI ANGGARAN BKAD</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr"/>
+      <c r="A2" s="7" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>Kolom</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>Tipe Data</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>Keterangan</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>Contoh</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>tahun</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>Angka (integer)</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>Tahun anggaran (4 digit)</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E4" s="9" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>nama_opd</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="9" t="inlineStr">
         <is>
           <t>Teks</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>Nama lengkap OPD</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E5" s="9" t="inlineStr">
         <is>
           <t>Badan Keuangan dan Aset Daerah (BKAD)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>penanggungjawab</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>Teks</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>Bidang penanggung jawab kegiatan</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E6" s="9" t="inlineStr">
         <is>
           <t>Sekretariat / Bidang Anggaran / Bidang Perbendaharaan</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>kode_rekening</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>Teks</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>Kode Rekening SIPD/SIMDA</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="E7" s="9" t="inlineStr">
         <is>
           <t>5.02.01.2.01.0001</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>jenis_belanja</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>Teks</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D8" s="9" t="inlineStr">
         <is>
           <t>Nama Sub-Kegiatan / Jenis Belanja</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E8" s="9" t="inlineStr">
         <is>
           <t>Penyusunan Dokumen Perencanaan Perangkat Daerah</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>bulan</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>Angka (1-12)</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D9" s="9" t="inlineStr">
         <is>
           <t>Bulan realisasi (1 = Jan, 12 = Des)</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="E9" s="9" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>pagu_anggaran</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>Angka (Rupiah)</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D10" s="9" t="inlineStr">
         <is>
           <t>Pagu anggaran Rupiah penuh (tanpa titik/koma)</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E10" s="9" t="inlineStr">
         <is>
           <t>16342500</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>realisasi</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>Angka (Rupiah)</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>Realisasi kumulatif Rupiah penuh s.d. bulan tersebut</t>
-        </is>
-      </c>
-      <c r="E11" s="8" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Nilai realisasi bulanan mentah Rupiah penuh pada bulan berkenaan</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
         <is>
           <t>2440000</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr"/>
+      <c r="A12" s="7" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="inlineStr">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>PENTING:</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>1. Jangan mengubah nama kolom (baris pertama) pada sheet 'Data Realisasi'</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>2. Data realisasi bersifat KUMULATIF per bulan</t>
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>2. Data realisasi diisi per bulan (mentah/non-kumulatif). Sistem Dashboard akan menghitung akumulasi secara otomatis</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>3. Pagu anggaran bernilai SAMA untuk semua bulan dalam 1 tahun per kegiatan</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>4. Hapus 3 baris contoh (baris abu-abu) sebelum mengisi data asli</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>5. Simpan file dalam format .xlsx</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr"/>
+      <c r="A19" s="7" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>DAFTAR BIDANG PENANGGUNG JAWAB:</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
+      <c r="A21" s="7" t="inlineStr">
         <is>
           <t>- Sekretariat</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
+      <c r="A22" s="7" t="inlineStr">
         <is>
           <t>- Bidang Anggaran</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="inlineStr">
+      <c r="A23" s="7" t="inlineStr">
         <is>
           <t>- Bidang Perbendaharaan</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
+      <c r="A24" s="7" t="inlineStr">
         <is>
           <t>- Bidang Akuntansi &amp; Pelaporan</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr">
+      <c r="A25" s="7" t="inlineStr">
         <is>
           <t>- Bidang Pengelolaan BMD</t>
         </is>

</xml_diff>

<commit_message>
chore: perbarui data dummy dan template upload pasca rollback
</commit_message>
<xml_diff>
--- a/data/template_upload.xlsx
+++ b/data/template_upload.xlsx
@@ -1,13 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Realisasi" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Petunjuk Pengisian" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Data Realisasi" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Petunjuk Pengisian" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,18 +18,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
@@ -82,27 +75,12 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -118,47 +96,43 @@
       <bottom style="thin">
         <color rgb="00D9D9D9"/>
       </bottom>
-      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -535,151 +509,151 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>tahun</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>nama_opd</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>penanggungjawab</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>kode_rekening</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>jenis_belanja</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>bulan</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>pagu_anggaran</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>realisasi</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="n">
+      <c r="A2" s="2" t="n">
         <v>2025</v>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Badan Keuangan dan Aset Daerah (BKAD)</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Sekretariat</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>5.02.01.2.01.0001</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Penyusunan Dokumen Perencanaan Perangkat Daerah</t>
         </is>
       </c>
-      <c r="F2" s="3" t="n">
+      <c r="F2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G2" s="5" t="n">
+      <c r="G2" s="4" t="n">
         <v>16342500</v>
       </c>
-      <c r="H2" s="5" t="n">
+      <c r="H2" s="4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n">
+      <c r="A3" s="2" t="n">
         <v>2025</v>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Badan Keuangan dan Aset Daerah (BKAD)</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Sekretariat</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>5.02.01.2.01.0001</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>Penyusunan Dokumen Perencanaan Perangkat Daerah</t>
         </is>
       </c>
-      <c r="F3" s="3" t="n">
+      <c r="F3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G3" s="5" t="n">
+      <c r="G3" s="4" t="n">
         <v>16342500</v>
       </c>
-      <c r="H3" s="5" t="n">
+      <c r="H3" s="4" t="n">
         <v>2440000</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n">
+      <c r="A4" s="2" t="n">
         <v>2025</v>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Badan Keuangan dan Aset Daerah (BKAD)</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Bidang Anggaran</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>5.02.02.2.01.0001</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Koordinasi dan Penyusunan KUA dan PPAS</t>
         </is>
       </c>
-      <c r="F4" s="3" t="n">
+      <c r="F4" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G4" s="5" t="n">
+      <c r="G4" s="4" t="n">
         <v>325936500</v>
       </c>
-      <c r="H4" s="5" t="n">
+      <c r="H4" s="4" t="n">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -700,343 +674,343 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>PETUNJUK PENGISIAN TEMPLATE DATA REALISASI ANGGARAN BKAD</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr"/>
+      <c r="A2" s="6" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>Kolom</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>Tipe Data</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>Keterangan</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>Contoh</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>tahun</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>Angka (integer)</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="8" t="inlineStr">
         <is>
           <t>Tahun anggaran (4 digit)</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>nama_opd</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>Teks</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>Nama lengkap OPD</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>Badan Keuangan dan Aset Daerah (BKAD)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>penanggungjawab</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>Teks</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>Bidang penanggung jawab kegiatan</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>Sekretariat / Bidang Anggaran / Bidang Perbendaharaan</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>kode_rekening</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>Teks</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>Kode Rekening SIPD/SIMDA</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>5.02.01.2.01.0001</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>jenis_belanja</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>Teks</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>Nama Sub-Kegiatan / Jenis Belanja</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E8" s="8" t="inlineStr">
         <is>
           <t>Penyusunan Dokumen Perencanaan Perangkat Daerah</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>bulan</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>Angka (1-12)</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>Bulan realisasi (1 = Jan, 12 = Des)</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="E9" s="8" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>pagu_anggaran</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>Angka (Rupiah)</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>Pagu anggaran Rupiah penuh (tanpa titik/koma)</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
+      <c r="E10" s="8" t="inlineStr">
         <is>
           <t>16342500</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>realisasi</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>Angka (Rupiah)</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>Nilai realisasi bulanan mentah Rupiah penuh pada bulan berkenaan</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr">
         <is>
           <t>2440000</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr"/>
+      <c r="A12" s="6" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>PENTING:</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>1. Jangan mengubah nama kolom (baris pertama) pada sheet 'Data Realisasi'</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>2. Data realisasi diisi per bulan (mentah/non-kumulatif). Sistem Dashboard akan menghitung akumulasi secara otomatis</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>3. Pagu anggaran bernilai SAMA untuk semua bulan dalam 1 tahun per kegiatan</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>4. Hapus 3 baris contoh (baris abu-abu) sebelum mengisi data asli</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>5. Simpan file dalam format .xlsx</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="inlineStr"/>
+      <c r="A19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="inlineStr">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>DAFTAR BIDANG PENANGGUNG JAWAB:</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>- Sekretariat</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="inlineStr">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>- Bidang Anggaran</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="inlineStr">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>- Bidang Perbendaharaan</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="inlineStr">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>- Bidang Akuntansi &amp; Pelaporan</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="inlineStr">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>- Bidang Pengelolaan BMD</t>
         </is>

</xml_diff>